<commit_message>
Agrega carga masiva de matriculas con plantilla Excel
</commit_message>
<xml_diff>
--- a/Aplicaciones/Gestion/plantillas_excel/plantilla_estudiantes.xlsx
+++ b/Aplicaciones/Gestion/plantillas_excel/plantilla_estudiantes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\UTC\8VO\TESIS\APLICACIÓN\Colegio\Aplicaciones\Gestion\plantillas_excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4C873CBB-8642-498C-9B3B-809A6721DF12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{076A7745-36AD-41D3-8002-4EE688503E6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,6 +44,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>OpenAI</author>
+    <author>PC</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000001000000}">
@@ -326,12 +327,65 @@
         </r>
       </text>
     </comment>
+    <comment ref="U1" authorId="1" shapeId="0" xr:uid="{AEC4BBBC-D88C-438E-94E4-9D5EBF80DFC1}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Campo obligatorio
+NOTA: Poner el nombre exactamente como esta registrado el curso</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="1" shapeId="0" xr:uid="{BBA0F9A5-2DE6-46C2-B323-89C56DC07346}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Campo obligatorio</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="1" shapeId="0" xr:uid="{B536F3B2-6F7A-418A-B8C9-9025E3ED8E57}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Opcional
+</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
   <si>
     <t>cedula</t>
   </si>
@@ -544,6 +598,15 @@
   </si>
   <si>
     <t>OTRA_NACIONALIDAD</t>
+  </si>
+  <si>
+    <t>curso_aprobado</t>
+  </si>
+  <si>
+    <t>institucion_procedencia</t>
+  </si>
+  <si>
+    <t>observacion_ingreso</t>
   </si>
 </sst>
 </file>
@@ -554,7 +617,7 @@
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -592,6 +655,27 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="4">
@@ -655,7 +739,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -674,6 +758,7 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -976,7 +1061,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T500"/>
+  <dimension ref="A1:W500"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.109375" customWidth="1"/>
@@ -994,9 +1079,12 @@
     <col min="15" max="15" width="14" customWidth="1"/>
     <col min="16" max="18" width="16" customWidth="1"/>
     <col min="19" max="20" width="22" customWidth="1"/>
+    <col min="21" max="21" width="23.33203125" customWidth="1"/>
+    <col min="22" max="22" width="29.44140625" customWidth="1"/>
+    <col min="23" max="23" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1057,8 +1145,17 @@
       <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="U1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6"/>
       <c r="B2" s="7"/>
       <c r="C2" s="7"/>
@@ -1078,79 +1175,82 @@
       <c r="R2" s="7"/>
       <c r="S2" s="7"/>
       <c r="T2" s="7"/>
-    </row>
-    <row r="3" spans="1:20" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="U2" s="7"/>
+      <c r="V2" s="7"/>
+    </row>
+    <row r="3" spans="1:23" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9"/>
       <c r="F3" s="8"/>
       <c r="H3" s="7"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="F5" s="3"/>
       <c r="O5" s="2"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" s="2"/>
       <c r="B6" s="2"/>
       <c r="F6" s="3"/>
       <c r="O6" s="2"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
       <c r="F7" s="3"/>
       <c r="O7" s="2"/>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="V7" s="10"/>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" s="2"/>
       <c r="B8" s="2"/>
       <c r="F8" s="3"/>
       <c r="O8" s="2"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A9" s="2"/>
       <c r="B9" s="2"/>
       <c r="F9" s="3"/>
       <c r="O9" s="2"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="F10" s="3"/>
       <c r="O10" s="2"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" s="2"/>
       <c r="B11" s="2"/>
       <c r="F11" s="3"/>
       <c r="O11" s="2"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" s="2"/>
       <c r="B12" s="2"/>
       <c r="F12" s="3"/>
       <c r="O12" s="2"/>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
       <c r="F13" s="3"/>
       <c r="O13" s="2"/>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" s="2"/>
       <c r="B14" s="2"/>
       <c r="F14" s="3"/>
       <c r="O14" s="2"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" s="2"/>
       <c r="B15" s="2"/>
       <c r="F15" s="3"/>
       <c r="O15" s="2"/>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" s="2"/>
       <c r="B16" s="2"/>
       <c r="F16" s="3"/>

</xml_diff>